<commit_message>
Commit after test case seggregation 04/02
</commit_message>
<xml_diff>
--- a/Config/Testcases.xlsx
+++ b/Config/Testcases.xlsx
@@ -6,6 +6,7 @@
     <sheet name="Testcases" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet2" sheetId="3" r:id="rId3"/>
+    <sheet name="Final" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -426,7 +427,7 @@
         <v>Check if the user can navigate to the ad hoc payment requests section of the web application.</v>
       </c>
       <c r="C2" t="str">
-        <v>True</v>
+        <v>No</v>
       </c>
       <c r="D2" t="str">
         <v>TestValidLogin</v>
@@ -1510,12 +1511,12 @@
         <v>VerifyApproveRejectAllButtons</v>
       </c>
       <c r="E94" t="str" xml:space="preserve">
-        <v xml:space="preserve">FAIL - Error: strict mode violation: Locator("text=Approvals") resolved to 3 elements:_x000d_
-    1) &lt;span class="MuiTypography-root MuiTypography-body1 MuiListItemText-primary css-fyswvn"&gt;Approvals&lt;/span&gt; aka GetByRole(AriaRole.Button, new() { Name = "Approvals" })_x000d_
-    2) &lt;h5 class="MuiTypography-root MuiTypography-h5 approvals-tittle css-6id74z"&gt;Ad-hoc payments - Approvals&lt;/h5&gt; aka GetByRole(AriaRole.Heading, new() { Name = "Ad-hoc payments - Approvals" })_x000d_
-    3) &lt;button role="tab" tabindex="-1" type="button" aria-selected="false" class="MuiButtonBase-root MuiTab-root MuiTab-labelIcon MuiTab-textColorPrimary ↵ tab ↵ horizontal ↵ inactive-tab↵ icon-with-text↵ ↵ icon-position-end↵ primary↵ css-1dliu7k"&gt;…&lt;/button&gt; aka GetByRole(AriaRole.Tab, new() { Name = "APPROVALS 99+" })_x000d_
-_x000d_
-Call log:_x000d_
+        <v xml:space="preserve">FAIL - Error: strict mode violation: Locator("text=Approvals") resolved to 3 elements:_x000d__x000d__x000d_
+    1) &lt;span class="MuiTypography-root MuiTypography-body1 MuiListItemText-primary css-fyswvn"&gt;Approvals&lt;/span&gt; aka GetByRole(AriaRole.Button, new() { Name = "Approvals" })_x000d__x000d__x000d_
+    2) &lt;h5 class="MuiTypography-root MuiTypography-h5 approvals-tittle css-6id74z"&gt;Ad-hoc payments - Approvals&lt;/h5&gt; aka GetByRole(AriaRole.Heading, new() { Name = "Ad-hoc payments - Approvals" })_x000d__x000d__x000d_
+    3) &lt;button role="tab" tabindex="-1" type="button" aria-selected="false" class="MuiButtonBase-root MuiTab-root MuiTab-labelIcon MuiTab-textColorPrimary ↵ tab ↵ horizontal ↵ inactive-tab↵ icon-with-text↵ ↵ icon-position-end↵ primary↵ css-1dliu7k"&gt;…&lt;/button&gt; aka GetByRole(AriaRole.Tab, new() { Name = "APPROVALS 99+" })_x000d__x000d__x000d_
+_x000d__x000d__x000d_
+Call log:_x000d__x000d__x000d_
   - waiting for Locator("text=Approvals")</v>
       </c>
     </row>
@@ -6142,4 +6143,3208 @@
     <ignoredError numberStoredAsText="1" sqref="A1:E382"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E191"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>TestCaseID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>TestCaseName</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Execute</v>
+      </c>
+      <c r="D1" t="str">
+        <v>MethodName</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Result_x000d_</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>190495</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Check if the "Login" button is displayed on the login page without user name and password field.</v>
+      </c>
+      <c r="C2" t="str">
+        <v>True</v>
+      </c>
+      <c r="D2" t="str">
+        <v>TestValidLogin</v>
+      </c>
+      <c r="E2" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>190496</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Check if clicking the "Login" button redirects to the Microsoft SSO login page.</v>
+      </c>
+      <c r="C3" t="str">
+        <v>True</v>
+      </c>
+      <c r="D3" t="str">
+        <v>TestValidLogin</v>
+      </c>
+      <c r="E3" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>190497</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Check if only the authorised list of users are allowed to login to the application</v>
+      </c>
+      <c r="C4" t="str">
+        <v>True</v>
+      </c>
+      <c r="D4" t="str">
+        <v>TestValidLogin</v>
+      </c>
+      <c r="E4" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>190498</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Check if the user not allowed to login with a incorrect username or password</v>
+      </c>
+      <c r="C5" t="str">
+        <v>True</v>
+      </c>
+      <c r="D5" t="str">
+        <v>TestValidLogin</v>
+      </c>
+      <c r="E5" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>190499</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Check if successful login redirects the user to the application’s homepage.</v>
+      </c>
+      <c r="C6" t="str">
+        <v>True</v>
+      </c>
+      <c r="D6" t="str">
+        <v>TestValidLogin</v>
+      </c>
+      <c r="E6" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>190506</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Check if the user could able to view the login page once the URL is entered._x000d_</v>
+      </c>
+      <c r="C7" t="str">
+        <v>True</v>
+      </c>
+      <c r="D7" t="str">
+        <v>TestValidLogin</v>
+      </c>
+      <c r="E7" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>190509</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Check if the user could able to successfully login to the application.</v>
+      </c>
+      <c r="C8" t="str">
+        <v>True</v>
+      </c>
+      <c r="D8" t="str">
+        <v>TestValidLogin</v>
+      </c>
+      <c r="E8" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>190511</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Check if the user is directed to the Ad-hoc payments landing page once logged in.</v>
+      </c>
+      <c r="C9" t="str">
+        <v>True</v>
+      </c>
+      <c r="D9" t="str">
+        <v>TestValidLogin</v>
+      </c>
+      <c r="E9" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>190523</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Check if the users could able to navigate to different pages easily._x000d_</v>
+      </c>
+      <c r="C10" t="str">
+        <v>True</v>
+      </c>
+      <c r="D10" t="str">
+        <v>TestValidLogin</v>
+      </c>
+      <c r="E10" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>190536</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Check if the user lands on the Ad-Hoc payments login page after logging in.</v>
+      </c>
+      <c r="C11" t="str">
+        <v>True</v>
+      </c>
+      <c r="D11" t="str">
+        <v>TestValidLogin</v>
+      </c>
+      <c r="E11" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>190537</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Check if the user can view and click the “Create New Request” button to initiate a new ad-hoc payment request.</v>
+      </c>
+      <c r="C12" t="str">
+        <v>No</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>190538</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Check if clicking the “Create Request” button displays the payment request form.</v>
+      </c>
+      <c r="C13" t="str">
+        <v>No</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>190540</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Check if the requested name and requested date fields are available at top right portion of the form._x000d_</v>
+      </c>
+      <c r="C14" t="str">
+        <v>No</v>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>190541</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Check if an alert message appears if the user tries to submit the form without filling any fields.</v>
+      </c>
+      <c r="C15" t="str">
+        <v>No</v>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>190542</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Check if the system highlights incomplete mandatory fields when the user attempts to submit the form without filling them.</v>
+      </c>
+      <c r="C16" t="str">
+        <v>No</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>190543</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Check if the form didn't allow the user to submit the request by entering the past date in payment due by date field._x000d_</v>
+      </c>
+      <c r="C17" t="str">
+        <v>No</v>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>190545</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Check if the beneficiary name field accepts upper case, lower case and numerics and allows up to 35 characters._x000d_</v>
+      </c>
+      <c r="C18" t="str">
+        <v>No</v>
+      </c>
+      <c r="D18" t="str">
+        <v>TestValidLogin</v>
+      </c>
+      <c r="E18" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>190546</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Check if the account number field accepts only 8 characters if the payment region is UK._x000d_</v>
+      </c>
+      <c r="C19" t="str">
+        <v>No</v>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>190547</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Check if the account number field accepts only 15 characters if the payment region is International._x000d_</v>
+      </c>
+      <c r="C20" t="str">
+        <v>No</v>
+      </c>
+      <c r="D20" t="str">
+        <v>TestValidLogin</v>
+      </c>
+      <c r="E20" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>190548</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Check if the IBAN field is not mandatory and the request can be submitted if it is not populated._x000d_</v>
+      </c>
+      <c r="C21" t="str">
+        <v>No</v>
+      </c>
+      <c r="D21" t="str">
+        <v>ApproveRequest</v>
+      </c>
+      <c r="E21" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>190549</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Check if the IBAN field accepts onlu 34 characters.</v>
+      </c>
+      <c r="C22" t="str">
+        <v>No</v>
+      </c>
+      <c r="D22" t="str">
+        <v>TestValidLogin</v>
+      </c>
+      <c r="E22" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>190550</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Check if the BIC field is not mandatory and the request can be submitted if it is not populated._x000d_</v>
+      </c>
+      <c r="C23" t="str">
+        <v>No</v>
+      </c>
+      <c r="D23" t="str">
+        <v>CreateNewRequest</v>
+      </c>
+      <c r="E23" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>190551</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Check if the BIC field accepts only 11 characters._x000d_</v>
+      </c>
+      <c r="C24" t="str">
+        <v>No</v>
+      </c>
+      <c r="D24" t="str">
+        <v>CreateNewRequest</v>
+      </c>
+      <c r="E24" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>190552</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Check if the system validates numeric fields to ensure only positive numbers are entered (e.g., Payment Amount)._x000d_</v>
+      </c>
+      <c r="C25" t="str">
+        <v>No</v>
+      </c>
+      <c r="D25" t="str">
+        <v>CreateNewRequest</v>
+      </c>
+      <c r="E25" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>190553</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Check if the Net value and Vat amount fields accepts upto 11 numerics._x000d_</v>
+      </c>
+      <c r="C26" t="str">
+        <v>No</v>
+      </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
+      <c r="E26" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>190557</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Check if the VAT Amount field enables if the VAT applicable field is selected "YES"._x000d_</v>
+      </c>
+      <c r="C27" t="str">
+        <v>No</v>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+      <c r="E27" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>190558</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Check if the VAT Amount field disables if the VAT applicable field is selected "No"._x000d_</v>
+      </c>
+      <c r="C28" t="str">
+        <v>No</v>
+      </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
+      <c r="E28" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>190559</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Check if the user can type in the dropdown field to fetch the values in the dropdown._x000d_</v>
+      </c>
+      <c r="C29" t="str">
+        <v>No</v>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
+      <c r="E29" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>190560</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Verify that the Nominal Code field allows a minimum of 5 and a maximum of 11 characters._x000d_</v>
+      </c>
+      <c r="C30" t="str">
+        <v>No</v>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>190561</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Verify that the Nominal Code must begin with the letter "C"._x000d_</v>
+      </c>
+      <c r="C31" t="str">
+        <v>No</v>
+      </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
+      <c r="E31" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>190562</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Verify that the Nominal Code allows both numeric and alphanumeric values._x000d_</v>
+      </c>
+      <c r="C32" t="str">
+        <v>No</v>
+      </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
+      <c r="E32" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>190563</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Verify that the Nominal Code field rejects values exceeding 11 characters._x000d_</v>
+      </c>
+      <c r="C33" t="str">
+        <v>No</v>
+      </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
+      <c r="E33" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>190564</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Check if the (Optional) text in the Cost Center field is removed.</v>
+      </c>
+      <c r="C34" t="str">
+        <v>No</v>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
+      <c r="E34" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>190565</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Check if the user could able to save the request even if the cost center field is not populated.</v>
+      </c>
+      <c r="C35" t="str">
+        <v>No</v>
+      </c>
+      <c r="D35" t="str">
+        <v>CreateNewRequest</v>
+      </c>
+      <c r="E35" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>190567</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Check if the form allows resubmission after the user corrects the errors.</v>
+      </c>
+      <c r="C36" t="str">
+        <v>No</v>
+      </c>
+      <c r="D36" t="str">
+        <v>CreateNewRequest</v>
+      </c>
+      <c r="E36" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>190568</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Check if the user could able to attach files through drag and drop and browse files.</v>
+      </c>
+      <c r="C37" t="str">
+        <v>No</v>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+      <c r="E37" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>190570</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Check if the user could able to upload file with size greater than the allowed limit.</v>
+      </c>
+      <c r="C38" t="str">
+        <v>No</v>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+      <c r="E38" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>190573</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Check if the system successfully submits the payment request when all validations pass.</v>
+      </c>
+      <c r="C39" t="str">
+        <v>No</v>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+      <c r="E39" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>190574</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Verify that payments above £250,000 automatically update the Payment Type to "CHAPS".</v>
+      </c>
+      <c r="C40" t="str">
+        <v>No</v>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+      <c r="E40" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>190575</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Verify that an alert is displayed when the Payment Type is changed to "CHAPS" due to the payment amount.</v>
+      </c>
+      <c r="C41" t="str">
+        <v>No</v>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
+      <c r="E41" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>190576</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Verify that the user cannot manually change the Payment Type once it is set to "CHAPS" automatically._x000d_</v>
+      </c>
+      <c r="C42" t="str">
+        <v>No</v>
+      </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
+      <c r="E42" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>190577</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Verify that payments of £250,000 or below allow manual Payment Type selection._x000d_</v>
+      </c>
+      <c r="C43" t="str">
+        <v>No</v>
+      </c>
+      <c r="D43" t="str">
+        <v/>
+      </c>
+      <c r="E43" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>190578</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Verify system behavior when a payment amount is updated from below £250,000 to above £250,000._x000d_</v>
+      </c>
+      <c r="C44" t="str">
+        <v>No</v>
+      </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
+      <c r="E44" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>190579</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Verify system behavior when a payment amount is reduced from above £250,000 to below.</v>
+      </c>
+      <c r="C45" t="str">
+        <v>No</v>
+      </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
+      <c r="E45" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>190580</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Verify that the Debit Account Currency field is enabled for user selection._x000d_</v>
+      </c>
+      <c r="C46" t="str">
+        <v>No</v>
+      </c>
+      <c r="D46" t="str">
+        <v>TestValidLogin</v>
+      </c>
+      <c r="E46" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>190581</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Verify that the default currency is preselected based on the predefined payable account settings._x000d_</v>
+      </c>
+      <c r="C47" t="str">
+        <v>No</v>
+      </c>
+      <c r="D47" t="str">
+        <v>ApproveRequest</v>
+      </c>
+      <c r="E47" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>190582</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Verify that users can modify and save the selected currency before submitting the payment._x000d_</v>
+      </c>
+      <c r="C48" t="str">
+        <v>No</v>
+      </c>
+      <c r="D48" t="str">
+        <v>ApproveRequest</v>
+      </c>
+      <c r="E48" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>190583</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Verify that the currency dropdown displays "GBP" at the top, followed by other currencies in alphabetical order._x000d_</v>
+      </c>
+      <c r="C49" t="str">
+        <v>No</v>
+      </c>
+      <c r="D49" t="str">
+        <v>ApproveRequest</v>
+      </c>
+      <c r="E49" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>190585</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Verify that users can quickly locate an account name in the structured dropdown.</v>
+      </c>
+      <c r="C50" t="str">
+        <v>No</v>
+      </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
+      <c r="E50" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>190586</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Check if a confirmation message “Ad-Hoc Payment Request Submitted Successfully” is displayed upon successful submission.</v>
+      </c>
+      <c r="C51" t="str">
+        <v>No</v>
+      </c>
+      <c r="D51" t="str">
+        <v/>
+      </c>
+      <c r="E51" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>190587</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Check if the user is redirected to the payment request grid page showing a summary of the submitted request.</v>
+      </c>
+      <c r="C52" t="str">
+        <v>No</v>
+      </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
+      <c r="E52" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>190588</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Check if the user could able to view the created payment request in the payment request grid.</v>
+      </c>
+      <c r="C53" t="str">
+        <v>No</v>
+      </c>
+      <c r="D53" t="str">
+        <v/>
+      </c>
+      <c r="E53" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>190590</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Check if the user can navigate to the adhoc payment view page by clicking on the request id.</v>
+      </c>
+      <c r="C54" t="str">
+        <v>No</v>
+      </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
+      <c r="E54" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>190591</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Check if the right pane has 3 different tabs "Request Details", "Attachment &amp; Info" and "Audit Log".</v>
+      </c>
+      <c r="C55" t="str">
+        <v>No</v>
+      </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
+      <c r="E55" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>190593</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Check if each entry in the request list includes relevant details provided during request creation.</v>
+      </c>
+      <c r="C56" t="str">
+        <v>No</v>
+      </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
+      <c r="E56" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>190594</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Check if the system displays documents attached to each ad hoc payment request in the "Attachments and Info" tab.</v>
+      </c>
+      <c r="C57" t="str">
+        <v>No</v>
+      </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
+      <c r="E57" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>190595</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Check if the system displays all input details provided during request creation for the selected payment request._x000d_</v>
+      </c>
+      <c r="C58" t="str">
+        <v>No</v>
+      </c>
+      <c r="D58" t="str">
+        <v>RejectRequest</v>
+      </c>
+      <c r="E58" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>190597</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Check if the system shows the rejection reason for requests that have been rejected._x000d_</v>
+      </c>
+      <c r="C59" t="str">
+        <v>No</v>
+      </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
+      <c r="E59" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>190600</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Check if the user can return to the request list by clicking the close button after viewing an individual request._x000d_</v>
+      </c>
+      <c r="C60" t="str">
+        <v>No</v>
+      </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
+      <c r="E60" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>190602</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Check if the user can navigate to the ad hoc payment requests section of the web application._x000d_</v>
+      </c>
+      <c r="C61" t="str">
+        <v>No</v>
+      </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
+      <c r="E61" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>190604</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Check if the user can identify and select a request to modify by clicking the "Edit" button._x000d_</v>
+      </c>
+      <c r="C62" t="str">
+        <v>No</v>
+      </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
+      <c r="E62" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>190605</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Check if the edit icon appears in the grid if the status of the payment request is "Pending" or "Rejected"._x000d_</v>
+      </c>
+      <c r="C63" t="str">
+        <v>No</v>
+      </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
+      <c r="E63" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>190606</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Check if the system allows access to the modification form when the request status is "Pending" or "Rejected."_x000d_</v>
+      </c>
+      <c r="C64" t="str">
+        <v>No</v>
+      </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
+      <c r="E64" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>190607</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Check if the user can edit the request by clicking on the "Edit Request" button in the view screen._x000d_</v>
+      </c>
+      <c r="C65" t="str">
+        <v>No</v>
+      </c>
+      <c r="D65" t="str">
+        <v/>
+      </c>
+      <c r="E65" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>190610</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Check if the user can modify editable fields in the form as needed._x000d_</v>
+      </c>
+      <c r="C66" t="str">
+        <v>No</v>
+      </c>
+      <c r="D66" t="str">
+        <v/>
+      </c>
+      <c r="E66" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>190611</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Check if the system performs mandatory field validation upon submission of the modified request._x000d_</v>
+      </c>
+      <c r="C67" t="str">
+        <v>No</v>
+      </c>
+      <c r="D67" t="str">
+        <v/>
+      </c>
+      <c r="E67" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>190613</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Check if the system highlights problematic fields and displays specific error messages if validation errors occur._x000d_</v>
+      </c>
+      <c r="C68" t="str">
+        <v>No</v>
+      </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
+      <c r="E68" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>190614</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Check if the user can correct validation errors based on the error messages provided._x000d_</v>
+      </c>
+      <c r="C69" t="str">
+        <v>No</v>
+      </c>
+      <c r="D69" t="str">
+        <v/>
+      </c>
+      <c r="E69" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>190615</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Check if the user can resubmit the modified request after correcting any validation errors._x000d_</v>
+      </c>
+      <c r="C70" t="str">
+        <v>No</v>
+      </c>
+      <c r="D70" t="str">
+        <v/>
+      </c>
+      <c r="E70" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>190616</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Check if the system successfully updates the request when all validations pass._x000d_</v>
+      </c>
+      <c r="C71" t="str">
+        <v>No</v>
+      </c>
+      <c r="D71" t="str">
+        <v/>
+      </c>
+      <c r="E71" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>190617</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Check if a confirmation message “Payment Request Updated Successfully” is displayed upon successful modification._x000d_</v>
+      </c>
+      <c r="C72" t="str">
+        <v>No</v>
+      </c>
+      <c r="D72" t="str">
+        <v/>
+      </c>
+      <c r="E72" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>190618</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Check if the user is able to navigate back to the list of payment requests after modification._x000d_</v>
+      </c>
+      <c r="C73" t="str">
+        <v>No</v>
+      </c>
+      <c r="D73" t="str">
+        <v/>
+      </c>
+      <c r="E73" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>190620</v>
+      </c>
+      <c r="B74" t="str">
+        <v>Check if the approver can log into the web application with approver privileges._x000d_</v>
+      </c>
+      <c r="C74" t="str">
+        <v>No</v>
+      </c>
+      <c r="D74" t="str">
+        <v/>
+      </c>
+      <c r="E74" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>190621</v>
+      </c>
+      <c r="B75" t="str">
+        <v>Check if the approver can navigate to the "Approvals" section from the main menu._x000d_</v>
+      </c>
+      <c r="C75" t="str">
+        <v>No</v>
+      </c>
+      <c r="D75" t="str">
+        <v/>
+      </c>
+      <c r="E75" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>190622</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Check if the system displays three tabs within the "Approvals" section: "Pending", "Approved" and "Rejected."_x000d_</v>
+      </c>
+      <c r="C76" t="str">
+        <v>No</v>
+      </c>
+      <c r="D76" t="str">
+        <v/>
+      </c>
+      <c r="E76" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>190623</v>
+      </c>
+      <c r="B77" t="str">
+        <v>Check if the approver can access the "Pending" tab._x000d_</v>
+      </c>
+      <c r="C77" t="str">
+        <v>No</v>
+      </c>
+      <c r="D77" t="str">
+        <v/>
+      </c>
+      <c r="E77" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>190628</v>
+      </c>
+      <c r="B78" t="str">
+        <v>Check if the approver can approve a request by clicking the "Approve" button._x000d_</v>
+      </c>
+      <c r="C78" t="str">
+        <v>No</v>
+      </c>
+      <c r="D78" t="str">
+        <v/>
+      </c>
+      <c r="E78" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>190629</v>
+      </c>
+      <c r="B79" t="str">
+        <v>Check if the system updates the request status to "Approved" upon approval._x000d_</v>
+      </c>
+      <c r="C79" t="str">
+        <v>No</v>
+      </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
+      <c r="E79" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>190630</v>
+      </c>
+      <c r="B80" t="str">
+        <v>Check if the approved request moves to the "Approved" tab after approval._x000d_</v>
+      </c>
+      <c r="C80" t="str">
+        <v>No</v>
+      </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
+      <c r="E80" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>190631</v>
+      </c>
+      <c r="B81" t="str">
+        <v>Check if the count of the tabs "Pending" and "Approved" are updated once the record is approved._x000d_</v>
+      </c>
+      <c r="C81" t="str">
+        <v>No</v>
+      </c>
+      <c r="D81" t="str">
+        <v/>
+      </c>
+      <c r="E81" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>190632</v>
+      </c>
+      <c r="B82" t="str">
+        <v>Check if the system sends a notification to the requester indicating their request has been approved._x000d_</v>
+      </c>
+      <c r="C82" t="str">
+        <v>No</v>
+      </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
+      <c r="E82" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>190633</v>
+      </c>
+      <c r="B83" t="str">
+        <v>Check if the approver can reject a request by clicking the "Reject" button._x000d_</v>
+      </c>
+      <c r="C83" t="str">
+        <v>No</v>
+      </c>
+      <c r="D83" t="str">
+        <v/>
+      </c>
+      <c r="E83" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>190634</v>
+      </c>
+      <c r="B84" t="str">
+        <v>Check if a field for entering a rejection reason is displayed when the approver clicks the "Reject" button._x000d_</v>
+      </c>
+      <c r="C84" t="str">
+        <v>No</v>
+      </c>
+      <c r="D84" t="str">
+        <v/>
+      </c>
+      <c r="E84" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>190635</v>
+      </c>
+      <c r="B85" t="str">
+        <v>Check if the rejection reason field requires the approver to enter a specific reason for rejection._x000d_</v>
+      </c>
+      <c r="C85" t="str">
+        <v>No</v>
+      </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
+      <c r="E85" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>190636</v>
+      </c>
+      <c r="B86" t="str">
+        <v>Check if the request moves to the "Rejected" tab with its status updated after being rejected._x000d_</v>
+      </c>
+      <c r="C86" t="str">
+        <v>No</v>
+      </c>
+      <c r="D86" t="str">
+        <v/>
+      </c>
+      <c r="E86" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>190637</v>
+      </c>
+      <c r="B87" t="str">
+        <v>Check if the count of the tabs "Pending" and "Rejected" are updated once the record is rejected._x000d_</v>
+      </c>
+      <c r="C87" t="str">
+        <v>No</v>
+      </c>
+      <c r="D87" t="str">
+        <v/>
+      </c>
+      <c r="E87" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>190638</v>
+      </c>
+      <c r="B88" t="str">
+        <v>Check if the system sends a notification to the requester with the rejection reason._x000d_</v>
+      </c>
+      <c r="C88" t="str">
+        <v>No</v>
+      </c>
+      <c r="D88" t="str">
+        <v/>
+      </c>
+      <c r="E88" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>190639</v>
+      </c>
+      <c r="B89" t="str">
+        <v>Check if the approver can navigate back to the "Pending" list after taking action on a request._x000d_</v>
+      </c>
+      <c r="C89" t="str">
+        <v>No</v>
+      </c>
+      <c r="D89" t="str">
+        <v/>
+      </c>
+      <c r="E89" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>190640</v>
+      </c>
+      <c r="B90" t="str">
+        <v>Check if the approver can seamlessly switch between the "Pending," "Approved," and "Rejected" tabs to view requests in each category._x000d_</v>
+      </c>
+      <c r="C90" t="str">
+        <v>No</v>
+      </c>
+      <c r="D90" t="str">
+        <v/>
+      </c>
+      <c r="E90" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>190641</v>
+      </c>
+      <c r="B91" t="str">
+        <v>Check if the user can log into the application and access the section for managing approved payment requests._x000d_</v>
+      </c>
+      <c r="C91" t="str">
+        <v>No</v>
+      </c>
+      <c r="D91" t="str">
+        <v/>
+      </c>
+      <c r="E91" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>190642</v>
+      </c>
+      <c r="B92" t="str">
+        <v>Check if the application displays a list of approved ad hoc payment requests along with the "Generate Files" button._x000d_</v>
+      </c>
+      <c r="C92" t="str">
+        <v>No</v>
+      </c>
+      <c r="D92" t="str">
+        <v/>
+      </c>
+      <c r="E92" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>190643</v>
+      </c>
+      <c r="B93" t="str">
+        <v>Check if there is a "Generated Files" column appears in the grid._x000d_</v>
+      </c>
+      <c r="C93" t="str">
+        <v>No</v>
+      </c>
+      <c r="D93" t="str">
+        <v/>
+      </c>
+      <c r="E93" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>190651</v>
+      </c>
+      <c r="B94" t="str">
+        <v>Check if the system generates a D365 file in the specified format with data from the selected requests._x000d_</v>
+      </c>
+      <c r="C94" t="str">
+        <v>No</v>
+      </c>
+      <c r="D94" t="str">
+        <v>VerifyApproveRejectAllButtons</v>
+      </c>
+      <c r="E94" t="str">
+        <v>FAIL - Error: strict mode violation: Locator("text=Approvals") resolved to 3 elements:_x000d_</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>190652</v>
+      </c>
+      <c r="B95" t="str">
+        <v>Check if a confirmation message “Files have been generated successfully” is displayed after the files are generated._x000d_</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>190659</v>
+      </c>
+      <c r="B96" t="str">
+        <v>Check if generated files in the Generated Files List can be downloaded by the user._x000d_</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>190698</v>
+      </c>
+      <c r="B97" t="str">
+        <v>Check if a Download button is available for each file entry in the Generated Files List screen._x000d_</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>190699</v>
+      </c>
+      <c r="B98" t="str">
+        <v>Check if clicking the Download button on the Generated Files List screen directly downloads the respective file in .csv format._x000d_</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>190704</v>
+      </c>
+      <c r="B99" t="str">
+        <v>Check if requests with the status "File Generated" are displayed in the Approved tab of the Approvals screen._x000d_</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>190705</v>
+      </c>
+      <c r="B100" t="str">
+        <v>Check if the user can select a request with "File Generated" status in the Approved tab to view its details._x000d_</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>190707</v>
+      </c>
+      <c r="B101" t="str">
+        <v>Check if each file entry in the detailed view has a Download button in the Approved tab._x000d_</v>
+      </c>
+      <c r="C101" t="str">
+        <v>No</v>
+      </c>
+      <c r="D101" t="str">
+        <v/>
+      </c>
+      <c r="E101" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>190708</v>
+      </c>
+      <c r="B102" t="str">
+        <v>Check if clicking the Download button in the detailed view of the Approved tab directly downloads the respective file in .csv format._x000d_</v>
+      </c>
+      <c r="C102" t="str">
+        <v>No</v>
+      </c>
+      <c r="D102" t="str">
+        <v/>
+      </c>
+      <c r="E102" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>190714</v>
+      </c>
+      <c r="B103" t="str">
+        <v>Check if each file entry includes an "Edit" button to modify its details._x000d_</v>
+      </c>
+      <c r="C103" t="str">
+        <v>No</v>
+      </c>
+      <c r="D103" t="str">
+        <v/>
+      </c>
+      <c r="E103" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>190715</v>
+      </c>
+      <c r="B104" t="str">
+        <v>Check if clicking on the edit icon opens a right side pane along with the file details._x000d_</v>
+      </c>
+      <c r="C104" t="str">
+        <v>No</v>
+      </c>
+      <c r="D104" t="str">
+        <v/>
+      </c>
+      <c r="E104" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>190716</v>
+      </c>
+      <c r="B105" t="str">
+        <v>Check if clicking the "Edit" button allows the user to update the Upload Status and Reference Number for the selected file._x000d_</v>
+      </c>
+      <c r="C105" t="str">
+        <v>No</v>
+      </c>
+      <c r="D105" t="str">
+        <v/>
+      </c>
+      <c r="E105" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>190717</v>
+      </c>
+      <c r="B106" t="str">
+        <v>Check if the Upload Status field provides "Yes" or "No" options for selection._x000d_</v>
+      </c>
+      <c r="C106" t="str">
+        <v>No</v>
+      </c>
+      <c r="D106" t="str">
+        <v/>
+      </c>
+      <c r="E106" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>190718</v>
+      </c>
+      <c r="B107" t="str">
+        <v>Check if the Reference Number field allows the user to enter or update the reference number for the selected file._x000d_</v>
+      </c>
+      <c r="C107" t="str">
+        <v>No</v>
+      </c>
+      <c r="D107" t="str">
+        <v/>
+      </c>
+      <c r="E107" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>190719</v>
+      </c>
+      <c r="B108" t="str">
+        <v>Check if the Ref.No field accepts only up to 15 characters and is alphanumerical._x000d_</v>
+      </c>
+      <c r="C108" t="str">
+        <v>No</v>
+      </c>
+      <c r="D108" t="str">
+        <v/>
+      </c>
+      <c r="E108" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>190720</v>
+      </c>
+      <c r="B109" t="str">
+        <v>Check if clicking the "Save" button saves the updated Upload Status and Reference Number._x000d_</v>
+      </c>
+      <c r="C109" t="str">
+        <v>No</v>
+      </c>
+      <c r="D109" t="str">
+        <v/>
+      </c>
+      <c r="E109" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>190721</v>
+      </c>
+      <c r="B110" t="str">
+        <v>Check if the system validates the Reference Number against criteria upon saving._x000d_</v>
+      </c>
+      <c r="C110" t="str">
+        <v>No</v>
+      </c>
+      <c r="D110" t="str">
+        <v/>
+      </c>
+      <c r="E110" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>190722</v>
+      </c>
+      <c r="B111" t="str">
+        <v>Check if an error message is displayed when the Reference Number fails validation._x000d_</v>
+      </c>
+      <c r="C111" t="str">
+        <v>No</v>
+      </c>
+      <c r="D111" t="str">
+        <v/>
+      </c>
+      <c r="E111" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>190723</v>
+      </c>
+      <c r="B112" t="str">
+        <v>Check if a confirmation message ("File ID:# updated successfully") is displayed upon successful update and save._x000d_</v>
+      </c>
+      <c r="C112" t="str">
+        <v>No</v>
+      </c>
+      <c r="D112" t="str">
+        <v/>
+      </c>
+      <c r="E112" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>190724</v>
+      </c>
+      <c r="B113" t="str">
+        <v>Check if the Generated Files List refreshes automatically to display the updated Upload Status and Reference Number._x000d_</v>
+      </c>
+      <c r="C113" t="str">
+        <v>No</v>
+      </c>
+      <c r="D113" t="str">
+        <v/>
+      </c>
+      <c r="E113" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>190725</v>
+      </c>
+      <c r="B114" t="str">
+        <v>Check if the user can view the updated details of the file after refreshing the Generated Files List._x000d_</v>
+      </c>
+      <c r="C114" t="str">
+        <v>No</v>
+      </c>
+      <c r="D114" t="str">
+        <v/>
+      </c>
+      <c r="E114" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>190726</v>
+      </c>
+      <c r="B115" t="str">
+        <v>Check if the approver can log into the web application with approver privileges._x000d_</v>
+      </c>
+      <c r="C115" t="str">
+        <v>No</v>
+      </c>
+      <c r="D115" t="str">
+        <v/>
+      </c>
+      <c r="E115" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>190729</v>
+      </c>
+      <c r="B116" t="str">
+        <v>Check if the approver can access the "Pending" tab._x000d_</v>
+      </c>
+      <c r="C116" t="str">
+        <v>No</v>
+      </c>
+      <c r="D116" t="str">
+        <v/>
+      </c>
+      <c r="E116" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>190730</v>
+      </c>
+      <c r="B117" t="str">
+        <v>Check if the system displays a list of payment requests Pending under the "Pending" tab._x000d_</v>
+      </c>
+      <c r="C117" t="str">
+        <v>No</v>
+      </c>
+      <c r="D117" t="str">
+        <v/>
+      </c>
+      <c r="E117" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>190731</v>
+      </c>
+      <c r="B118" t="str">
+        <v>Check if a checkbox is available next to each payment request in the "Pending" list for selection._x000d_</v>
+      </c>
+      <c r="C118" t="str">
+        <v>No</v>
+      </c>
+      <c r="D118" t="str">
+        <v/>
+      </c>
+      <c r="E118" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>190732</v>
+      </c>
+      <c r="B119" t="str">
+        <v>Check if a “Select All” checkbox is provided to select all requests in the list at once._x000d_</v>
+      </c>
+      <c r="C119" t="str">
+        <v>No</v>
+      </c>
+      <c r="D119" t="str">
+        <v/>
+      </c>
+      <c r="E119" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>190733</v>
+      </c>
+      <c r="B120" t="str">
+        <v>Check if the approver can individually select multiple requests using checkboxes._x000d_</v>
+      </c>
+      <c r="C120" t="str">
+        <v>No</v>
+      </c>
+      <c r="D120" t="str">
+        <v/>
+      </c>
+      <c r="E120" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>190734</v>
+      </c>
+      <c r="B121" t="str">
+        <v>Check if the approver can select all requests using the “Select All” checkbox._x000d_</v>
+      </c>
+      <c r="C121" t="str">
+        <v>No</v>
+      </c>
+      <c r="D121" t="str">
+        <v/>
+      </c>
+      <c r="E121" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>190735</v>
+      </c>
+      <c r="B122" t="str">
+        <v>Check if the "Approve All" and "Reject All" buttons appear if the user selects more than one request._x000d_</v>
+      </c>
+      <c r="C122" t="str">
+        <v>No</v>
+      </c>
+      <c r="D122" t="str">
+        <v>TestValidLogin</v>
+      </c>
+      <c r="E122" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>190736</v>
+      </c>
+      <c r="B123" t="str">
+        <v>Check if the approver can perform a bulk approval action by selecting multiple requests and clicking the "Approve All" button._x000d_</v>
+      </c>
+      <c r="C123" t="str">
+        <v>No</v>
+      </c>
+      <c r="D123" t="str">
+        <v>CreateNewRequest</v>
+      </c>
+      <c r="E123" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>190737</v>
+      </c>
+      <c r="B124" t="str">
+        <v>Check if each selected request is moved to the "Approved" tab after bulk approval._x000d_</v>
+      </c>
+      <c r="C124" t="str">
+        <v>No</v>
+      </c>
+      <c r="D124" t="str">
+        <v/>
+      </c>
+      <c r="E124" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>190738</v>
+      </c>
+      <c r="B125" t="str">
+        <v>Check if the status of each selected request is updated to "Approved" after bulk approval._x000d_</v>
+      </c>
+      <c r="C125" t="str">
+        <v>No</v>
+      </c>
+      <c r="D125" t="str">
+        <v/>
+      </c>
+      <c r="E125" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>190739</v>
+      </c>
+      <c r="B126" t="str">
+        <v>Check if notifications are sent to each requester for the approved requests with the message “Your payment request titled [Request Title] has been approved.”_x000d_</v>
+      </c>
+      <c r="C126" t="str">
+        <v>No</v>
+      </c>
+      <c r="D126" t="str">
+        <v/>
+      </c>
+      <c r="E126" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>190740</v>
+      </c>
+      <c r="B127" t="str">
+        <v>Check if the approver can perform a bulk rejection action by selecting multiple requests and clicking the "Reject All" button._x000d_</v>
+      </c>
+      <c r="C127" t="str">
+        <v>No</v>
+      </c>
+      <c r="D127" t="str">
+        <v/>
+      </c>
+      <c r="E127" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>190741</v>
+      </c>
+      <c r="B128" t="str">
+        <v>Check if a dialogue box prompts the approver to input a rejection reason when the "Reject All" button is clicked in bulk mode._x000d_</v>
+      </c>
+      <c r="C128" t="str">
+        <v>No</v>
+      </c>
+      <c r="D128" t="str">
+        <v/>
+      </c>
+      <c r="E128" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>190742</v>
+      </c>
+      <c r="B129" t="str">
+        <v>Check if the approver can input rejection reasons for each request being rejected in the dialogue box._x000d_</v>
+      </c>
+      <c r="C129" t="str">
+        <v>No</v>
+      </c>
+      <c r="D129" t="str">
+        <v/>
+      </c>
+      <c r="E129" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>190743</v>
+      </c>
+      <c r="B130" t="str">
+        <v>Check if each selected request is moved to the "Rejected" tab after bulk rejection._x000d_</v>
+      </c>
+      <c r="C130" t="str">
+        <v>No</v>
+      </c>
+      <c r="D130" t="str">
+        <v/>
+      </c>
+      <c r="E130" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>190744</v>
+      </c>
+      <c r="B131" t="str">
+        <v>Check if the status of each selected request is updated to "Rejected" after bulk rejection._x000d_</v>
+      </c>
+      <c r="C131" t="str">
+        <v>No</v>
+      </c>
+      <c r="D131" t="str">
+        <v/>
+      </c>
+      <c r="E131" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>190745</v>
+      </c>
+      <c r="B132" t="str">
+        <v>Check if notifications are sent to each requester for the rejected requests with the message “Your payment request titled [Request Title] has been rejected. Reason: [Rejection Reason].”_x000d_</v>
+      </c>
+      <c r="C132" t="str">
+        <v>No</v>
+      </c>
+      <c r="D132" t="str">
+        <v/>
+      </c>
+      <c r="E132" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>190746</v>
+      </c>
+      <c r="B133" t="str">
+        <v>Check if the approver can return to the "Pending" tab after completing a bulk action._x000d_</v>
+      </c>
+      <c r="C133" t="str">
+        <v>No</v>
+      </c>
+      <c r="D133" t="str">
+        <v/>
+      </c>
+      <c r="E133" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>190747</v>
+      </c>
+      <c r="B134" t="str">
+        <v>Check if the approver can navigate between the "Pending," "Approved," and "Rejected" tabs to view requests in each category after a bulk action._x000d_</v>
+      </c>
+      <c r="C134" t="str">
+        <v>No</v>
+      </c>
+      <c r="D134" t="str">
+        <v/>
+      </c>
+      <c r="E134" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>190748</v>
+      </c>
+      <c r="B135" t="str">
+        <v>Check if the "Export" button is visible and enabled on the "Adhoc Requests &gt; Approvals" page._x000d_</v>
+      </c>
+      <c r="C135" t="str">
+        <v>No</v>
+      </c>
+      <c r="D135" t="str">
+        <v/>
+      </c>
+      <c r="E135" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>190766</v>
+      </c>
+      <c r="B136" t="str">
+        <v>Check if the "Upload Requests" button is available in the Landing View of Ad-hoc Payments &gt; Requests._x000d_</v>
+      </c>
+      <c r="C136" t="str">
+        <v>No</v>
+      </c>
+      <c r="D136" t="str">
+        <v/>
+      </c>
+      <c r="E136" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>190767</v>
+      </c>
+      <c r="B137" t="str">
+        <v>Check if clicking the "Upload Requests" button opens a file upload dialogue._x000d_</v>
+      </c>
+      <c r="C137" t="str">
+        <v>No</v>
+      </c>
+      <c r="D137" t="str">
+        <v/>
+      </c>
+      <c r="E137" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>190768</v>
+      </c>
+      <c r="B138" t="str">
+        <v>Check if the system allows selecting and uploading files in supported formats (xlsx, xls, csv) only._x000d_</v>
+      </c>
+      <c r="C138" t="str">
+        <v>No</v>
+      </c>
+      <c r="D138" t="str">
+        <v/>
+      </c>
+      <c r="E138" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>190769</v>
+      </c>
+      <c r="B139" t="str">
+        <v>Check if the system restricts the file size to a maximum of 5MB._x000d_</v>
+      </c>
+      <c r="C139" t="str">
+        <v>No</v>
+      </c>
+      <c r="D139" t="str">
+        <v/>
+      </c>
+      <c r="E139" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>190771</v>
+      </c>
+      <c r="B140" t="str">
+        <v>Check if the system validates the file type and size upon upload._x000d_</v>
+      </c>
+      <c r="C140" t="str">
+        <v>No</v>
+      </c>
+      <c r="D140" t="str">
+        <v/>
+      </c>
+      <c r="E140" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>190786</v>
+      </c>
+      <c r="B141" t="str">
+        <v>Check if appropriate error messages and confirmations appear for different validation scenarios, ensuring clarity and user guidance._x000d_</v>
+      </c>
+      <c r="C141" t="str">
+        <v>No</v>
+      </c>
+      <c r="D141" t="str">
+        <v/>
+      </c>
+      <c r="E141" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>190806</v>
+      </c>
+      <c r="B142" t="str">
+        <v>Check if user is able to navigate to the Generated Files dashboard from the Ad-hoc Payments module._x000d_</v>
+      </c>
+      <c r="C142" t="str">
+        <v>No</v>
+      </c>
+      <c r="D142" t="str">
+        <v/>
+      </c>
+      <c r="E142" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>190807</v>
+      </c>
+      <c r="B143" t="str">
+        <v>Check if user is able to view list of payment requests by clicking on a specific File ID._x000d_</v>
+      </c>
+      <c r="C143" t="str">
+        <v>No</v>
+      </c>
+      <c r="D143" t="str">
+        <v/>
+      </c>
+      <c r="E143" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="str">
+        <v>190808</v>
+      </c>
+      <c r="B144" t="str">
+        <v>Check if each payment request in the list displays relevant details._x000d_</v>
+      </c>
+      <c r="C144" t="str">
+        <v>No</v>
+      </c>
+      <c r="D144" t="str">
+        <v/>
+      </c>
+      <c r="E144" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="str">
+        <v>190809</v>
+      </c>
+      <c r="B145" t="str">
+        <v>Check if the “REJECT” button is visible for each request in the list._x000d_</v>
+      </c>
+      <c r="C145" t="str">
+        <v>No</v>
+      </c>
+      <c r="D145" t="str">
+        <v/>
+      </c>
+      <c r="E145" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="str">
+        <v>190810</v>
+      </c>
+      <c r="B146" t="str">
+        <v>Check if clicking the “REJECT” button opens a side panel with request details._x000d_</v>
+      </c>
+      <c r="C146" t="str">
+        <v>No</v>
+      </c>
+      <c r="D146" t="str">
+        <v/>
+      </c>
+      <c r="E146" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="str">
+        <v>190811</v>
+      </c>
+      <c r="B147" t="str">
+        <v>Check if user is able to enter a rejection reason in the comment box._x000d_</v>
+      </c>
+      <c r="C147" t="str">
+        <v>No</v>
+      </c>
+      <c r="D147" t="str">
+        <v/>
+      </c>
+      <c r="E147" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="str">
+        <v>190812</v>
+      </c>
+      <c r="B148" t="str">
+        <v>Check if user is able to submit the rejection after entering a comment._x000d_</v>
+      </c>
+      <c r="C148" t="str">
+        <v>No</v>
+      </c>
+      <c r="D148" t="str">
+        <v/>
+      </c>
+      <c r="E148" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="str">
+        <v>190813</v>
+      </c>
+      <c r="B149" t="str">
+        <v>Check if rejection confirmation message is displayed after rejecting a request._x000d_</v>
+      </c>
+      <c r="C149" t="str">
+        <v>No</v>
+      </c>
+      <c r="D149" t="str">
+        <v/>
+      </c>
+      <c r="E149" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="str">
+        <v>190814</v>
+      </c>
+      <c r="B150" t="str">
+        <v>Check if the request status updates to “Rejected” after successful rejection._x000d_</v>
+      </c>
+      <c r="C150" t="str">
+        <v>No</v>
+      </c>
+      <c r="D150" t="str">
+        <v/>
+      </c>
+      <c r="E150" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="str">
+        <v>190815</v>
+      </c>
+      <c r="B151" t="str">
+        <v>Check if rejected request is excluded from further processing as per the standard workflow._x000d_</v>
+      </c>
+      <c r="C151" t="str">
+        <v>No</v>
+      </c>
+      <c r="D151" t="str">
+        <v/>
+      </c>
+      <c r="E151" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="str">
+        <v>190816</v>
+      </c>
+      <c r="B152" t="str">
+        <v>Check if audit trail is updated after a request is rejected._x000d_</v>
+      </c>
+      <c r="C152" t="str">
+        <v>No</v>
+      </c>
+      <c r="D152" t="str">
+        <v/>
+      </c>
+      <c r="E152" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="str">
+        <v>190817</v>
+      </c>
+      <c r="B153" t="str">
+        <v>Check if previously approved requests are associated with newly generated files after rejection._x000d_</v>
+      </c>
+      <c r="C153" t="str">
+        <v>No</v>
+      </c>
+      <c r="D153" t="str">
+        <v/>
+      </c>
+      <c r="E153" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="str">
+        <v>190818</v>
+      </c>
+      <c r="B154" t="str">
+        <v>Check if generated files are shown under a separate tab within a request._x000d_</v>
+      </c>
+      <c r="C154" t="str">
+        <v>No</v>
+      </c>
+      <c r="D154" t="str">
+        <v/>
+      </c>
+      <c r="E154" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="str">
+        <v>190819</v>
+      </c>
+      <c r="B155" t="str">
+        <v>Check if Notes section displays the value entered during rejection._x000d_</v>
+      </c>
+      <c r="C155" t="str">
+        <v>No</v>
+      </c>
+      <c r="D155" t="str">
+        <v/>
+      </c>
+      <c r="E155" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="str">
+        <v>190820</v>
+      </c>
+      <c r="B156" t="str">
+        <v>Check if rejection is blocked when the comment box is left empty._x000d_</v>
+      </c>
+      <c r="C156" t="str">
+        <v>No</v>
+      </c>
+      <c r="D156" t="str">
+        <v/>
+      </c>
+      <c r="E156" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="str">
+        <v>190821</v>
+      </c>
+      <c r="B157" t="str">
+        <v>Check if user can cancel the rejection process using the close button or cancel option._x000d_</v>
+      </c>
+      <c r="C157" t="str">
+        <v>No</v>
+      </c>
+      <c r="D157" t="str">
+        <v/>
+      </c>
+      <c r="E157" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="str">
+        <v>190822</v>
+      </c>
+      <c r="B158" t="str">
+        <v>Check if the Edit Request page is accessible for requests with Pending Approval status._x000d_</v>
+      </c>
+      <c r="C158" t="str">
+        <v>No</v>
+      </c>
+      <c r="D158" t="str">
+        <v/>
+      </c>
+      <c r="E158" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="str">
+        <v>190823</v>
+      </c>
+      <c r="B159" t="str">
+        <v>Check if the Edit Request page is accessible for requests with Rejected status._x000d_</v>
+      </c>
+      <c r="C159" t="str">
+        <v>No</v>
+      </c>
+      <c r="D159" t="str">
+        <v/>
+      </c>
+      <c r="E159" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="str">
+        <v>190824</v>
+      </c>
+      <c r="B160" t="str">
+        <v>Check if the user is able to successfully save changes for a request in Pending Approval status._x000d_</v>
+      </c>
+      <c r="C160" t="str">
+        <v>No</v>
+      </c>
+      <c r="D160" t="str">
+        <v/>
+      </c>
+      <c r="E160" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="str">
+        <v>190825</v>
+      </c>
+      <c r="B161" t="str">
+        <v>Check if the user is able to successfully save changes for a request in Rejected status._x000d_</v>
+      </c>
+      <c r="C161" t="str">
+        <v>No</v>
+      </c>
+      <c r="D161" t="str">
+        <v/>
+      </c>
+      <c r="E161" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="str">
+        <v>190826</v>
+      </c>
+      <c r="B162" t="str">
+        <v>Check if the system prevents saving changes when the request status is Approved._x000d_</v>
+      </c>
+      <c r="C162" t="str">
+        <v>No</v>
+      </c>
+      <c r="D162" t="str">
+        <v/>
+      </c>
+      <c r="E162" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="str">
+        <v>190827</v>
+      </c>
+      <c r="B163" t="str">
+        <v>Check if the system prevents saving changes for requests in any other final state (e.g., Closed)._x000d_</v>
+      </c>
+      <c r="C163" t="str">
+        <v>No</v>
+      </c>
+      <c r="D163" t="str">
+        <v/>
+      </c>
+      <c r="E163" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="str">
+        <v>190828</v>
+      </c>
+      <c r="B164" t="str">
+        <v>Check if the system validates the current request status in real-time before saving._x000d_</v>
+      </c>
+      <c r="C164" t="str">
+        <v>No</v>
+      </c>
+      <c r="D164" t="str">
+        <v/>
+      </c>
+      <c r="E164" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>190864</v>
+      </c>
+      <c r="B165" t="str">
+        <v>Check if Notes section displays existing notes in descending order of timestamp_x000d_</v>
+      </c>
+      <c r="C165" t="str">
+        <v>No</v>
+      </c>
+      <c r="D165" t="str">
+        <v/>
+      </c>
+      <c r="E165" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="str">
+        <v>190865</v>
+      </c>
+      <c r="B166" t="str">
+        <v>Check if each note displays the author name and timestamp_x000d_</v>
+      </c>
+      <c r="C166" t="str">
+        <v>No</v>
+      </c>
+      <c r="D166" t="str">
+        <v/>
+      </c>
+      <c r="E166" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="str">
+        <v>190866</v>
+      </c>
+      <c r="B167" t="str">
+        <v>Check if user is able to add a new note with valid content_x000d_</v>
+      </c>
+      <c r="C167" t="str">
+        <v>No</v>
+      </c>
+      <c r="D167" t="str">
+        <v/>
+      </c>
+      <c r="E167" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="str">
+        <v>190867</v>
+      </c>
+      <c r="B168" t="str">
+        <v>Check if user is restricted from adding notes with more than 1000 characters_x000d_</v>
+      </c>
+      <c r="C168" t="str">
+        <v>No</v>
+      </c>
+      <c r="D168" t="str">
+        <v/>
+      </c>
+      <c r="E168" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="str">
+        <v>190868</v>
+      </c>
+      <c r="B169" t="str">
+        <v>Check if only the author of a note can delete it_x000d_</v>
+      </c>
+      <c r="C169" t="str">
+        <v>No</v>
+      </c>
+      <c r="D169" t="str">
+        <v/>
+      </c>
+      <c r="E169" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="str">
+        <v>190869</v>
+      </c>
+      <c r="B170" t="str">
+        <v>Check if deletion of a note is recorded in the Audit Log_x000d_</v>
+      </c>
+      <c r="C170" t="str">
+        <v>No</v>
+      </c>
+      <c r="D170" t="str">
+        <v/>
+      </c>
+      <c r="E170" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="str">
+        <v>190870</v>
+      </c>
+      <c r="B171" t="str">
+        <v>Check if "Rejection Notes" are displayed in the Notes section with appropriate title_x000d_</v>
+      </c>
+      <c r="C171" t="str">
+        <v>No</v>
+      </c>
+      <c r="D171" t="str">
+        <v/>
+      </c>
+      <c r="E171" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="str">
+        <v>190871</v>
+      </c>
+      <c r="B172" t="str">
+        <v>Check if "Rejection Notes" cannot be deleted by any user_x000d_</v>
+      </c>
+      <c r="C172" t="str">
+        <v>No</v>
+      </c>
+      <c r="D172" t="str">
+        <v/>
+      </c>
+      <c r="E172" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="str">
+        <v>190872</v>
+      </c>
+      <c r="B173" t="str">
+        <v>Check if audit log captures all note addition, deletion, and rejection note actions_x000d_</v>
+      </c>
+      <c r="C173" t="str">
+        <v>No</v>
+      </c>
+      <c r="D173" t="str">
+        <v/>
+      </c>
+      <c r="E173" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="str">
+        <v>190873</v>
+      </c>
+      <c r="B174" t="str">
+        <v>Check if notes are displayed consistently across sessions_x000d_</v>
+      </c>
+      <c r="C174" t="str">
+        <v>No</v>
+      </c>
+      <c r="D174" t="str">
+        <v/>
+      </c>
+      <c r="E174" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="str">
+        <v>190874</v>
+      </c>
+      <c r="B175" t="str">
+        <v>Check if note input field resets after successfully adding a note_x000d_</v>
+      </c>
+      <c r="C175" t="str">
+        <v>No</v>
+      </c>
+      <c r="D175" t="str">
+        <v/>
+      </c>
+      <c r="E175" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="str">
+        <v/>
+      </c>
+      <c r="B176" t="str">
+        <v>Check if the user is able to successfully save changes for a request in Pending Approval status</v>
+      </c>
+      <c r="C176" t="str">
+        <v>No</v>
+      </c>
+      <c r="D176" t="str">
+        <v/>
+      </c>
+      <c r="E176" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="str">
+        <v>113987</v>
+      </c>
+      <c r="B177" t="str">
+        <v>Check if the user is able to successfully save changes for a request in Rejected status</v>
+      </c>
+      <c r="C177" t="str">
+        <v>No</v>
+      </c>
+      <c r="D177" t="str">
+        <v/>
+      </c>
+      <c r="E177" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="str">
+        <v>113988</v>
+      </c>
+      <c r="B178" t="str">
+        <v>Check if the system prevents saving changes when the request status is Approved</v>
+      </c>
+      <c r="C178" t="str">
+        <v>No</v>
+      </c>
+      <c r="D178" t="str">
+        <v/>
+      </c>
+      <c r="E178" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="str">
+        <v>113989</v>
+      </c>
+      <c r="B179" t="str">
+        <v>Check if the system prevents saving changes for requests in any other final state (e.g., Closed)</v>
+      </c>
+      <c r="C179" t="str">
+        <v>No</v>
+      </c>
+      <c r="D179" t="str">
+        <v/>
+      </c>
+      <c r="E179" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="str">
+        <v>113990</v>
+      </c>
+      <c r="B180" t="str">
+        <v>Check if the system validates the current request status in real-time before saving</v>
+      </c>
+      <c r="C180" t="str">
+        <v>No</v>
+      </c>
+      <c r="D180" t="str">
+        <v/>
+      </c>
+      <c r="E180" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>114026</v>
+      </c>
+      <c r="B181" t="str">
+        <v>Check if Notes section displays existing notes in descending order of timestamp</v>
+      </c>
+      <c r="C181" t="str">
+        <v>No</v>
+      </c>
+      <c r="D181" t="str">
+        <v/>
+      </c>
+      <c r="E181" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>114027</v>
+      </c>
+      <c r="B182" t="str">
+        <v>Check if each note displays the author name and timestamp</v>
+      </c>
+      <c r="C182" t="str">
+        <v>No</v>
+      </c>
+      <c r="D182" t="str">
+        <v/>
+      </c>
+      <c r="E182" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>114028</v>
+      </c>
+      <c r="B183" t="str">
+        <v>Check if user is able to add a new note with valid content</v>
+      </c>
+      <c r="C183" t="str">
+        <v>No</v>
+      </c>
+      <c r="D183" t="str">
+        <v/>
+      </c>
+      <c r="E183" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>114029</v>
+      </c>
+      <c r="B184" t="str">
+        <v>Check if user is restricted from adding notes with more than 1000 characters</v>
+      </c>
+      <c r="C184" t="str">
+        <v>No</v>
+      </c>
+      <c r="D184" t="str">
+        <v/>
+      </c>
+      <c r="E184" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>114030</v>
+      </c>
+      <c r="B185" t="str">
+        <v>Check if only the author of a note can delete it</v>
+      </c>
+      <c r="C185" t="str">
+        <v>No</v>
+      </c>
+      <c r="D185" t="str">
+        <v/>
+      </c>
+      <c r="E185" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>114031</v>
+      </c>
+      <c r="B186" t="str">
+        <v>Check if deletion of a note is recorded in the Audit Log</v>
+      </c>
+      <c r="C186" t="str">
+        <v>No</v>
+      </c>
+      <c r="D186" t="str">
+        <v/>
+      </c>
+      <c r="E186" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>114032</v>
+      </c>
+      <c r="B187" t="str">
+        <v>Check if "Rejection Notes" are displayed in the Notes section with appropriate title</v>
+      </c>
+      <c r="C187" t="str">
+        <v>No</v>
+      </c>
+      <c r="D187" t="str">
+        <v/>
+      </c>
+      <c r="E187" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>114033</v>
+      </c>
+      <c r="B188" t="str">
+        <v>Check if "Rejection Notes" cannot be deleted by any user</v>
+      </c>
+      <c r="C188" t="str">
+        <v>No</v>
+      </c>
+      <c r="D188" t="str">
+        <v/>
+      </c>
+      <c r="E188" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="str">
+        <v>114034</v>
+      </c>
+      <c r="B189" t="str">
+        <v>Check if audit log captures all note addition, deletion, and rejection note actions</v>
+      </c>
+      <c r="C189" t="str">
+        <v>No</v>
+      </c>
+      <c r="D189" t="str">
+        <v/>
+      </c>
+      <c r="E189" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="str">
+        <v>114035</v>
+      </c>
+      <c r="B190" t="str">
+        <v>Check if notes are displayed consistently across sessions</v>
+      </c>
+      <c r="C190" t="str">
+        <v>No</v>
+      </c>
+      <c r="D190" t="str">
+        <v/>
+      </c>
+      <c r="E190" t="str">
+        <v>_x000d_</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>114036</v>
+      </c>
+      <c r="B191" t="str">
+        <v>Check if note input field resets after successfully adding a note</v>
+      </c>
+      <c r="C191" t="str">
+        <v>No</v>
+      </c>
+      <c r="D191" t="str">
+        <v/>
+      </c>
+      <c r="E191" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E191"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>